<commit_message>
Set SN6505 to DNP for Trenz production
</commit_message>
<xml_diff>
--- a/manufacturing reports/BOM/BOM_xlsx-S001.xlsx
+++ b/manufacturing reports/BOM/BOM_xlsx-S001.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projekte\UltraZohm\Work_Altium\ultrazohm_carrierboard\manufacturing reports\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9F0184A6-4A51-4670-A3E5-DFDFD405429B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9F26293-C77B-4A27-AA2B-88847F8B16FE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{B0EAF6A4-B44E-436D-BF7F-E1E212ADBE6E}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="10215" xr2:uid="{8FBB6709-519B-46C8-8DCD-976A5305C973}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_xlsx-S001" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1524" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1507" uniqueCount="537">
   <si>
     <t>AN</t>
   </si>
@@ -1582,21 +1582,6 @@
   </si>
   <si>
     <t>TPS54260DGQR</t>
-  </si>
-  <si>
-    <t>31503</t>
-  </si>
-  <si>
-    <t>U9A, U9B, U21, U29</t>
-  </si>
-  <si>
-    <t>(cs) SN6505BDBVT</t>
-  </si>
-  <si>
-    <t>SOT23-6</t>
-  </si>
-  <si>
-    <t>SOT95P280X145-6N</t>
   </si>
   <si>
     <t>31504</t>
@@ -2029,8 +2014,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3929F2F-8D4E-4425-BACC-FC4FE39EDF5D}">
-  <dimension ref="A1:R95"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{530C0C18-A93D-48EF-B81D-F1831050FF7E}">
+  <dimension ref="A1:R94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
@@ -6923,7 +6908,7 @@
         <v>518</v>
       </c>
       <c r="B91" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>519</v>
@@ -6950,7 +6935,7 @@
         <v>25</v>
       </c>
       <c r="K91" s="2" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="L91" s="2" t="s">
         <v>26</v>
@@ -7027,159 +7012,103 @@
         <v>22</v>
       </c>
       <c r="R92" s="2" t="s">
-        <v>22</v>
+        <v>528</v>
       </c>
     </row>
     <row r="93" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B93" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>531</v>
+        <v>142</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>22</v>
       </c>
       <c r="H93" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="I93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="L93" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="M93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="N93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="O93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="P93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q93" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R93" s="2" t="s">
         <v>532</v>
-      </c>
-      <c r="I93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J93" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K93" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L93" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="P93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q93" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="R93" s="2" t="s">
-        <v>533</v>
       </c>
     </row>
     <row r="94" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="B94" s="1">
+        <v>1</v>
+      </c>
+      <c r="C94" s="2" t="s">
         <v>534</v>
       </c>
-      <c r="B94" s="1">
-        <v>3</v>
-      </c>
-      <c r="C94" s="2" t="s">
+      <c r="D94" s="2" t="s">
         <v>535</v>
       </c>
-      <c r="D94" s="2" t="s">
-        <v>536</v>
-      </c>
       <c r="E94" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G94" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="G94" s="1"/>
       <c r="H94" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="I94" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="I94" s="1"/>
       <c r="J94" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="K94" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="K94" s="1"/>
       <c r="L94" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="M94" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="N94" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="O94" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="P94" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q94" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="M94" s="1"/>
+      <c r="N94" s="1"/>
+      <c r="O94" s="1"/>
+      <c r="P94" s="1"/>
+      <c r="Q94" s="1"/>
       <c r="R94" s="2" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="95" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
-        <v>538</v>
-      </c>
-      <c r="B95" s="1">
-        <v>1</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>539</v>
-      </c>
-      <c r="D95" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="E95" s="2" t="s">
-        <v>540</v>
-      </c>
-      <c r="F95" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="G95" s="1"/>
-      <c r="H95" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="I95" s="1"/>
-      <c r="J95" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="K95" s="1"/>
-      <c r="L95" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M95" s="1"/>
-      <c r="N95" s="1"/>
-      <c r="O95" s="1"/>
-      <c r="P95" s="1"/>
-      <c r="Q95" s="1"/>
-      <c r="R95" s="2" t="s">
-        <v>541</v>
+        <v>536</v>
       </c>
     </row>
   </sheetData>

</xml_diff>